<commit_message>
feat: add dataSolicitacao, historicoPrazo, sort and zeroed categories
</commit_message>
<xml_diff>
--- a/public/data/problemas_v2.xlsx
+++ b/public/data/problemas_v2.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafael.oliveira\Desktop\dashboard-ti\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CFCC707-423E-4E58-9C51-01405DA04DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02E6133-981F-4E08-9D4B-656F469113D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base de Dados" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Base de Dados'!$A$1:$N$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Base de Dados'!$A$1:$P$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="119">
   <si>
     <t>Unidade</t>
   </si>
@@ -388,6 +388,12 @@
   </si>
   <si>
     <t>Urgência e Emergencia</t>
+  </si>
+  <si>
+    <t>Histórico de Prazo</t>
+  </si>
+  <si>
+    <t>Data de Solicitação</t>
   </si>
 </sst>
 </file>
@@ -454,7 +460,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -476,6 +482,9 @@
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -783,7 +792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -798,11 +807,13 @@
     <col min="10" max="10" width="31.42578125" customWidth="1"/>
     <col min="11" max="11" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="22" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.42578125" customWidth="1"/>
-    <col min="14" max="14" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="13.42578125" customWidth="1"/>
+    <col min="15" max="15" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -840,13 +851,19 @@
         <v>91</v>
       </c>
       <c r="M1" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -879,14 +896,16 @@
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="7">
+      <c r="M2" s="8"/>
+      <c r="N2" s="7">
         <v>46212</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="7"/>
+      <c r="P2" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -919,14 +938,16 @@
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="7">
+      <c r="M3" s="2"/>
+      <c r="N3" s="7">
         <v>46212</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="7"/>
+      <c r="P3" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>49</v>
       </c>
@@ -959,14 +980,16 @@
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
-      <c r="M4" s="7">
+      <c r="M4" s="2"/>
+      <c r="N4" s="7">
         <v>46203</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="O4" s="7"/>
+      <c r="P4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>49</v>
       </c>
@@ -999,14 +1022,16 @@
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
-      <c r="M5" s="7">
+      <c r="M5" s="2"/>
+      <c r="N5" s="7">
         <v>46197</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="O5" s="7"/>
+      <c r="P5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>49</v>
       </c>
@@ -1039,14 +1064,16 @@
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-      <c r="M6" s="7">
+      <c r="M6" s="2"/>
+      <c r="N6" s="7">
         <v>46197</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="7"/>
+      <c r="P6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>52</v>
       </c>
@@ -1079,14 +1106,16 @@
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
-      <c r="M7" s="7">
+      <c r="M7" s="1"/>
+      <c r="N7" s="7">
         <v>46212</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="O7" s="7"/>
+      <c r="P7" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>52</v>
       </c>
@@ -1121,14 +1150,16 @@
       <c r="L8" s="6">
         <v>10000</v>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="6"/>
+      <c r="N8" s="7">
         <v>46203</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="O8" s="7"/>
+      <c r="P8" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
@@ -1165,14 +1196,16 @@
       <c r="L9" s="6">
         <v>68850.600000000006</v>
       </c>
-      <c r="M9" s="7">
+      <c r="M9" s="6"/>
+      <c r="N9" s="7">
         <v>46203</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="O9" s="7"/>
+      <c r="P9" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
@@ -1207,14 +1240,16 @@
         <v>34300</v>
       </c>
       <c r="L10" s="2"/>
-      <c r="M10" s="7">
+      <c r="M10" s="2"/>
+      <c r="N10" s="7">
         <v>46212</v>
       </c>
-      <c r="N10" s="1" t="s">
+      <c r="O10" s="7"/>
+      <c r="P10" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
@@ -1251,10 +1286,12 @@
       <c r="L11" s="6">
         <v>7777.4</v>
       </c>
-      <c r="M11" s="1"/>
+      <c r="M11" s="6"/>
       <c r="N11" s="1"/>
-    </row>
-    <row r="12" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+    </row>
+    <row r="12" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
@@ -1291,14 +1328,16 @@
       <c r="L12" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="M12" s="7">
+      <c r="M12" s="4"/>
+      <c r="N12" s="7">
         <v>46197</v>
       </c>
-      <c r="N12" s="1" t="s">
+      <c r="O12" s="7"/>
+      <c r="P12" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
@@ -1331,14 +1370,16 @@
       </c>
       <c r="K13" s="4"/>
       <c r="L13" s="1"/>
-      <c r="M13" s="7">
+      <c r="M13" s="1"/>
+      <c r="N13" s="7">
         <v>46203</v>
       </c>
-      <c r="N13" s="1" t="s">
+      <c r="O13" s="7"/>
+      <c r="P13" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>59</v>
       </c>
@@ -1371,14 +1412,16 @@
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="1"/>
-      <c r="M14" s="7">
+      <c r="M14" s="1"/>
+      <c r="N14" s="7">
         <v>46207</v>
       </c>
-      <c r="N14" s="1" t="s">
+      <c r="O14" s="7"/>
+      <c r="P14" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>60</v>
       </c>
@@ -1411,14 +1454,16 @@
       </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
-      <c r="M15" s="7">
+      <c r="M15" s="2"/>
+      <c r="N15" s="7">
         <v>46222</v>
       </c>
-      <c r="N15" s="1" t="s">
+      <c r="O15" s="7"/>
+      <c r="P15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>60</v>
       </c>
@@ -1455,14 +1500,16 @@
       <c r="L16" s="6">
         <v>500</v>
       </c>
-      <c r="M16" s="1" t="s">
+      <c r="M16" s="6"/>
+      <c r="N16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="N16" s="1" t="s">
+      <c r="O16" s="1"/>
+      <c r="P16" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>58</v>
       </c>
@@ -1495,14 +1542,16 @@
       </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
-      <c r="M17" s="7">
+      <c r="M17" s="6"/>
+      <c r="N17" s="7">
         <v>46203</v>
       </c>
-      <c r="N17" s="1" t="s">
+      <c r="O17" s="7"/>
+      <c r="P17" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>58</v>
       </c>
@@ -1535,10 +1584,12 @@
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="6"/>
-      <c r="M18" s="1"/>
+      <c r="M18" s="6"/>
       <c r="N18" s="1"/>
-    </row>
-    <row r="19" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+    </row>
+    <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>99</v>
       </c>
@@ -1571,14 +1622,16 @@
       </c>
       <c r="K19" s="4"/>
       <c r="L19" s="1"/>
-      <c r="M19" s="7">
+      <c r="M19" s="1"/>
+      <c r="N19" s="7">
         <v>46212</v>
       </c>
-      <c r="N19" s="1" t="s">
+      <c r="O19" s="7"/>
+      <c r="P19" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>99</v>
       </c>
@@ -1611,14 +1664,16 @@
       </c>
       <c r="K20" s="4"/>
       <c r="L20" s="1"/>
-      <c r="M20" s="7">
+      <c r="M20" s="1"/>
+      <c r="N20" s="7">
         <v>46203</v>
       </c>
-      <c r="N20" s="1" t="s">
+      <c r="O20" s="7"/>
+      <c r="P20" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>57</v>
       </c>
@@ -1655,14 +1710,16 @@
       <c r="L21" s="6">
         <v>500</v>
       </c>
-      <c r="M21" s="7">
+      <c r="M21" s="6"/>
+      <c r="N21" s="7">
         <v>46203</v>
       </c>
-      <c r="N21" s="1" t="s">
+      <c r="O21" s="7"/>
+      <c r="P21" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>56</v>
       </c>
@@ -1695,12 +1752,14 @@
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="6"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1" t="s">
+      <c r="M22" s="6"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>56</v>
       </c>
@@ -1733,12 +1792,14 @@
       </c>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1" t="s">
+      <c r="M23" s="6"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>63</v>
       </c>
@@ -1771,12 +1832,14 @@
       </c>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1" t="s">
+      <c r="M24" s="4"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>63</v>
       </c>
@@ -1809,13 +1872,15 @@
       </c>
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1" t="s">
+      <c r="M25" s="4"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N25" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P25" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: add Hospital Municipal Cubatão occurrences
</commit_message>
<xml_diff>
--- a/public/data/problemas_v2.xlsx
+++ b/public/data/problemas_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafael.oliveira\Desktop\dashboard-ti\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02E6133-981F-4E08-9D4B-656F469113D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A2E053-7711-4CC7-B2B8-177FE4D9DA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="140">
   <si>
     <t>Unidade</t>
   </si>
@@ -394,6 +394,69 @@
   </si>
   <si>
     <t>Data de Solicitação</t>
+  </si>
+  <si>
+    <t>Hospital Municipal de Cubatão</t>
+  </si>
+  <si>
+    <t>Diretoria</t>
+  </si>
+  <si>
+    <t>Cobertura Wi‑Fi insuficiente</t>
+  </si>
+  <si>
+    <t>Limitação operacional e mobilidade</t>
+  </si>
+  <si>
+    <t>Implantação de 20 Access Points</t>
+  </si>
+  <si>
+    <t>TI/Alta gestão</t>
+  </si>
+  <si>
+    <t>Projeto estruturado</t>
+  </si>
+  <si>
+    <t>6500/mês</t>
+  </si>
+  <si>
+    <t>Ausência de monitoramento de impressão</t>
+  </si>
+  <si>
+    <t>Impressão</t>
+  </si>
+  <si>
+    <t>Médio</t>
+  </si>
+  <si>
+    <t>Custos elevados e falta de controle</t>
+  </si>
+  <si>
+    <t>Implantar solução de gestão de impressão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI </t>
+  </si>
+  <si>
+    <t>Recomendado</t>
+  </si>
+  <si>
+    <t>2000/mês</t>
+  </si>
+  <si>
+    <t>Necessidade de revisão da autonomia dos nobreaks</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Risco à continuidade operacional</t>
+  </si>
+  <si>
+    <t>Realizar testes e dimensionamento elétrico</t>
+  </si>
+  <si>
+    <t>Planejado</t>
   </si>
 </sst>
 </file>
@@ -792,7 +855,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -802,7 +865,7 @@
     <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41" customWidth="1"/>
     <col min="9" max="9" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="31.42578125" customWidth="1"/>
     <col min="11" max="11" width="16.5703125" bestFit="1" customWidth="1"/>
@@ -1879,6 +1942,142 @@
         <v>14</v>
       </c>
     </row>
+    <row r="26" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="L26" s="4">
+        <v>22000</v>
+      </c>
+      <c r="M26" s="4"/>
+      <c r="N26" s="7">
+        <v>46257</v>
+      </c>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="L27" s="4">
+        <v>8000</v>
+      </c>
+      <c r="M27" s="4"/>
+      <c r="N27" s="7">
+        <v>46288</v>
+      </c>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4">
+        <v>8000</v>
+      </c>
+      <c r="M28" s="4"/>
+      <c r="N28" s="7">
+        <v>46226</v>
+      </c>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P25" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: replace duration text with real dates in Wi-Fi PI rows
- Data de Solicitação: "45 dias"/"50 dias" -> 01/07/2026 (UPA São Raimundo
  Nonato e CD Picos)
- Prazo inicial: "20 dias" -> 20/07/2026 (UPA São Raimundo Nonato)

Não há mais texto em campo de data, então a ordenação por prazo volta a
funcionar corretamente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/problemas_v2.xlsx
+++ b/public/data/problemas_v2.xlsx
@@ -1216,11 +1216,11 @@
       <c r="L19">
         <v>1000</v>
       </c>
-      <c r="M19" t="str">
-        <v>45 dias</v>
-      </c>
-      <c r="N19" t="str">
-        <v>20 dias</v>
+      <c r="M19">
+        <v>46204</v>
+      </c>
+      <c r="N19">
+        <v>46223</v>
       </c>
       <c r="P19" t="str">
         <v>Alta</v>
@@ -1260,8 +1260,8 @@
       <c r="K20">
         <v>42883.44</v>
       </c>
-      <c r="M20" t="str">
-        <v>50 dias</v>
+      <c r="M20">
+        <v>46204</v>
       </c>
       <c r="N20">
         <v>46203</v>

</xml_diff>

<commit_message>
data: update problemas dataset from Dashboard_Tecnologia_UE e Ambulatorial, remove incomplete rows
Removidas 3 linhas sem Categoria/Problema (CD Uruçui, CD Campo Maior, CD São Raimundo Nonato).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PbwaadC7tdswGRPeytYBEr
</commit_message>
<xml_diff>
--- a/public/data/problemas_v2.xlsx
+++ b/public/data/problemas_v2.xlsx
@@ -5,9 +5,6 @@
   <sheets>
     <sheet name="Base de Dados" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Base de Dados'!A1:P33</definedName>
-  </definedNames>
 </workbook>
 </file>
 
@@ -37,7 +34,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="\R\$\ #,##0.00;[Red]\(\R\$\ #,##0.00\);\-"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -401,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -453,7 +450,7 @@
         <v>Prioridade</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
         <v>PS Santana</v>
       </c>
@@ -476,13 +473,13 @@
         <v>Impacto na produtividade</v>
       </c>
       <c r="H2" t="str">
-        <v>Substituir equipamentos</v>
+        <v>Concluir substituição dos equipamentos remanescentes junto ao fornecedor e validar desempenho dos novos ativos.</v>
       </c>
       <c r="I2" t="str">
-        <v>TI/Fornecedor</v>
+        <v>Multisuport</v>
       </c>
       <c r="J2" t="str">
-        <v>Em andamento processo de troca. 10 de 50.</v>
+        <v>Em andamento: 10 de 43 equipamentos substituídos.</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -494,11 +491,10 @@
         <v>46052</v>
       </c>
       <c r="N2">
-        <v>46212</v>
-      </c>
-      <c r="O2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Multisuport - Jul/2026_x000d_
-Multisuport - Set/2026</v>
+        <v>46204</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Substituição em andamento junto à Multisuport. Quantitativo validado no plano: 10 de 43.</v>
       </c>
       <c r="P2" t="str">
         <v>Alta</v>
@@ -527,13 +523,13 @@
         <v>Indisponibilidade</v>
       </c>
       <c r="H3" t="str">
-        <v>Notificação de prestador - Prefeitura</v>
+        <v>Monitorar comportamento dos links após a implantação do terceiro circuito de internet e manter tratativas junto à DTIC.</v>
       </c>
       <c r="I3" t="str">
-        <v>DTIC - Prefeitura</v>
+        <v>DTIC Prefeitura</v>
       </c>
       <c r="J3" t="str">
-        <v>Em análise técnica entre TI SBCD e Dtic</v>
+        <v>Em análise técnica.</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -541,8 +537,11 @@
       <c r="L3">
         <v>0</v>
       </c>
+      <c r="M3">
+        <v>46052</v>
+      </c>
       <c r="N3">
-        <v>46197</v>
+        <v>46174</v>
       </c>
       <c r="O3" t="str">
         <v>Instalado o 3º link da TIM (SBCD)</v>
@@ -551,7 +550,7 @@
         <v>Alta</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
+    <row r="4">
       <c r="A4" t="str">
         <v>UPA Jaçanã</v>
       </c>
@@ -574,13 +573,13 @@
         <v>Impacto na produtividade</v>
       </c>
       <c r="H4" t="str">
-        <v>Substituir equipamentos</v>
+        <v>Retomar tratativas com fornecedor para conclusão da troca dos equipamentos pendentes.</v>
       </c>
       <c r="I4" t="str">
-        <v>TI/Fornecedor</v>
+        <v>Multisuport</v>
       </c>
       <c r="J4" t="str">
-        <v>Trocas de equipamentos fornecedor. Processo parado</v>
+        <v>Parcialmente executado: 10 de 50 equipamentos substituídos. Aguardando retomada pelo fornecedor.</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -592,11 +591,10 @@
         <v>46052</v>
       </c>
       <c r="N4">
-        <v>46212</v>
-      </c>
-      <c r="O4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Multisuport - Jul/2026_x000d_
-Multisuport - Set/2026</v>
+        <v>46204</v>
+      </c>
+      <c r="O4" t="str">
+        <v>10 de 50 equipamentos substituídos. Aguardando retomada do fornecedor.</v>
       </c>
       <c r="P4" t="str">
         <v>Alta</v>
@@ -625,13 +623,13 @@
         <v>Queda operacional</v>
       </c>
       <c r="H5" t="str">
-        <v>Ampliar cobertura</v>
+        <v>Realizar análise de cobertura e apresentar proposta de ampliação da rede sem fio.</v>
       </c>
       <c r="I5" t="str">
-        <v>DTIC - Prefeitura</v>
+        <v>DTIC Prefeitura</v>
       </c>
       <c r="J5" t="str">
-        <v>Em análise técnica entre TI SBCD e Dtic</v>
+        <v>Em análise técnica.</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -639,8 +637,14 @@
       <c r="L5">
         <v>0</v>
       </c>
+      <c r="M5">
+        <v>46052</v>
+      </c>
       <c r="N5">
-        <v>46203</v>
+        <v>46174</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
       </c>
       <c r="P5" t="str">
         <v>Alta</v>
@@ -669,16 +673,25 @@
         <v>Indisponibilidade</v>
       </c>
       <c r="H6" t="str">
-        <v>Notificação de prestador - Prefeitura</v>
+        <v>Monitorar comportamento dos links após a implantação do terceiro circuito de internet e manter tratativas junto à DTIC.</v>
       </c>
       <c r="I6" t="str">
-        <v>DTIC - Prefeitura</v>
+        <v>DTIC Prefeitura</v>
       </c>
       <c r="J6" t="str">
-        <v>Em análise técnica entre TI SBCD e Dtic</v>
+        <v>Em análise técnica.</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>46052</v>
       </c>
       <c r="N6">
-        <v>46197</v>
+        <v>46266</v>
       </c>
       <c r="O6" t="str">
         <v>Instalado o 3º link da TIM (SBCD)</v>
@@ -698,7 +711,7 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D7" t="str">
-        <v>PCs patrimoniados do CRI com baixo desempenho</v>
+        <v>Computadores com baixo desempenho</v>
       </c>
       <c r="E7" t="str">
         <v>Hardware</v>
@@ -710,16 +723,28 @@
         <v>Impacto na produtividade</v>
       </c>
       <c r="H7" t="str">
-        <v>Necessidade de substituição</v>
+        <v>Elaborar levantamento técnico e plano de renovação do parque computacional.</v>
       </c>
       <c r="I7" t="str">
         <v>Alta Gestão</v>
       </c>
       <c r="J7" t="str">
-        <v>Necessidade de investimento para trocas</v>
-      </c>
-      <c r="N7">
-        <v>46212</v>
+        <v>Aguardando aprovação orçamentária.</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Entre R$ 25.000 à R$ 30.000</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>45962</v>
+      </c>
+      <c r="N7" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O7" t="str">
+        <v xml:space="preserve">Levantamento inicial para troca de 100 equipamentos </v>
       </c>
       <c r="P7" t="str">
         <v>Média</v>
@@ -748,22 +773,28 @@
         <v>Queda operacional</v>
       </c>
       <c r="H8" t="str">
-        <v>Ampliar cobertura</v>
+        <v>Elaborar projeto de expansão da cobertura sem fio e aprovação orçamentária.</v>
       </c>
       <c r="I8" t="str">
-        <v>TI/Alta Gestão</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J8" t="str">
-        <v>Necessidade de investimento para ampliação de controle</v>
-      </c>
-      <c r="K8" t="str">
-        <v xml:space="preserve"> </v>
+        <v>Aguardando aprovação orçamentária.</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
       </c>
       <c r="L8">
         <v>10000</v>
       </c>
-      <c r="N8">
-        <v>46203</v>
+      <c r="M8">
+        <v>45962</v>
+      </c>
+      <c r="N8" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O8" t="str">
+        <v/>
       </c>
       <c r="P8" t="str">
         <v>Alta</v>
@@ -780,7 +811,7 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D9" t="str">
-        <v>Emails corporativos</v>
+        <v>E-mails corporativos</v>
       </c>
       <c r="E9" t="str">
         <v>Emails</v>
@@ -792,22 +823,28 @@
         <v>Comunicação operacional</v>
       </c>
       <c r="H9" t="str">
-        <v>Necessidade de contratação dos serviços com a Microsoft</v>
+        <v>Formalizar contratação das licenças Microsoft e iniciar implantação das contas corporativas.</v>
       </c>
       <c r="I9" t="str">
-        <v>TI/Alta Gestão</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J9" t="str">
-        <v>Necessidade de investimento para aquisição de licenças</v>
+        <v>Aguardando aprovação orçamentária.</v>
       </c>
       <c r="K9">
-        <v>5737.55</v>
+        <v>6534.51</v>
       </c>
       <c r="L9">
         <v>68850.6</v>
       </c>
-      <c r="N9">
-        <v>46203</v>
+      <c r="M9">
+        <v>45962</v>
+      </c>
+      <c r="N9" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
       </c>
       <c r="P9" t="str">
         <v>Média</v>
@@ -824,42 +861,48 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D10" t="str">
-        <v>Risco ambiental</v>
+        <v>Antivírus</v>
       </c>
       <c r="E10" t="str">
-        <v>Infraestrutura</v>
+        <v>Segurança</v>
       </c>
       <c r="F10" t="str">
         <v>Crítico</v>
       </c>
       <c r="G10" t="str">
-        <v>Dano físico</v>
+        <v>Riscos de acessos</v>
       </c>
       <c r="H10" t="str">
-        <v>Adequar ambiente</v>
+        <v>Adquirir e implantar licenças corporativas com monitoramento centralizado.</v>
       </c>
       <c r="I10" t="str">
-        <v>TI</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J10" t="str">
-        <v>Edital realizado e substituido equipamentos</v>
+        <v>Aguardando aprovação orçamentária.</v>
       </c>
       <c r="K10">
-        <v>34300</v>
-      </c>
-      <c r="N10">
-        <v>45964</v>
+        <v>700</v>
+      </c>
+      <c r="L10">
+        <v>8400</v>
+      </c>
+      <c r="M10">
+        <v>45962</v>
+      </c>
+      <c r="N10" t="str">
+        <v>A definir</v>
       </c>
       <c r="O10" t="str">
-        <v>Finalizado em 11/2025</v>
+        <v/>
       </c>
       <c r="P10" t="str">
-        <v>Alta</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>AME Andradina</v>
+        <v>AME Promissão</v>
       </c>
       <c r="B11" t="str">
         <v>São Paulo</v>
@@ -880,19 +923,31 @@
         <v>Riscos de acessos</v>
       </c>
       <c r="H11" t="str">
-        <v>Implantação de licenças de antivírus</v>
+        <v>Contratação e implantação de solução corporativa de proteção de endpoints.</v>
       </c>
       <c r="I11" t="str">
-        <v>TI/Alta Gestão</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J11" t="str">
-        <v>Necessidade de investimento em aquisição de licenças</v>
+        <v>Aguardando aprovação orçamentária.</v>
       </c>
       <c r="K11">
-        <v>463.75</v>
+        <v>331.25</v>
       </c>
       <c r="L11">
-        <v>5565</v>
+        <v>3975</v>
+      </c>
+      <c r="M11">
+        <v>45962</v>
+      </c>
+      <c r="N11" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -906,31 +961,43 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D12" t="str">
-        <v>Antivírus</v>
+        <v>Link de redundância</v>
       </c>
       <c r="E12" t="str">
-        <v>Segurança</v>
+        <v>Rede</v>
       </c>
       <c r="F12" t="str">
         <v>Crítico</v>
       </c>
       <c r="G12" t="str">
-        <v>Riscos de acessos</v>
+        <v>Parada total</v>
       </c>
       <c r="H12" t="str">
-        <v>Implantação de licenças de antivírus</v>
+        <v>Contratar link redundante via satélite para contingência operacional.</v>
       </c>
       <c r="I12" t="str">
-        <v>TI/Alta Gestão</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J12" t="str">
-        <v>Necessidade de investimento em aquisição de licenças</v>
-      </c>
-      <c r="K12">
-        <v>331.25</v>
-      </c>
-      <c r="L12">
-        <v>3975</v>
+        <v>Aguardando aprovação orçamentária.</v>
+      </c>
+      <c r="K12" t="str">
+        <v>R$ 685 até R$ 1.235,00/mês</v>
+      </c>
+      <c r="L12" t="str">
+        <v>R$ 3.000,00 até R$ 5.000,00</v>
+      </c>
+      <c r="M12">
+        <v>45962</v>
+      </c>
+      <c r="N12" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v>Alta</v>
       </c>
     </row>
     <row r="13">
@@ -944,7 +1011,7 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D13" t="str">
-        <v>Rompimento fibra</v>
+        <v>Falhas de Wi-Fi</v>
       </c>
       <c r="E13" t="str">
         <v>Rede</v>
@@ -953,25 +1020,31 @@
         <v>Crítico</v>
       </c>
       <c r="G13" t="str">
-        <v>Parada total</v>
+        <v>Instabilidade</v>
       </c>
       <c r="H13" t="str">
-        <v>Implantar redundância via satélite para mudança de rota</v>
+        <v>Substituir equipamentos e ampliar cobertura da rede sem fio.</v>
       </c>
       <c r="I13" t="str">
-        <v>TI</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J13" t="str">
-        <v>Necessidade de investimento em link redundante</v>
-      </c>
-      <c r="K13" t="str">
-        <v>R$ 685 até R$ 1.235,00/mês</v>
+        <v>Aguardando aprovação orçamentária.</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
       </c>
       <c r="L13" t="str">
-        <v>R$ 3.000,00 até R$ 5.000,00</v>
-      </c>
-      <c r="N13">
-        <v>46197</v>
+        <v>R$ 15.000 a R$ 20.000</v>
+      </c>
+      <c r="M13">
+        <v>45962</v>
+      </c>
+      <c r="N13" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O13" t="str">
+        <v/>
       </c>
       <c r="P13" t="str">
         <v>Alta</v>
@@ -988,28 +1061,40 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D14" t="str">
-        <v>Falhas de Wi-Fi</v>
+        <v>Telemedicina</v>
       </c>
       <c r="E14" t="str">
-        <v>Rede</v>
+        <v>Sistema</v>
       </c>
       <c r="F14" t="str">
         <v>Crítico</v>
       </c>
       <c r="G14" t="str">
-        <v>Instabilidade</v>
+        <v>impacto operacional</v>
       </c>
       <c r="H14" t="str">
-        <v>Expandir cobertura</v>
+        <v>Manter o ambiente de telemedicina implantado e concluir a validação da integração operacional com a unidade.</v>
       </c>
       <c r="I14" t="str">
-        <v>TI</v>
+        <v xml:space="preserve">TI </v>
       </c>
       <c r="J14" t="str">
-        <v>Necessidade de investimento para troca de equipamentos</v>
+        <v>Concluído</v>
+      </c>
+      <c r="K14">
+        <v>895</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>46113</v>
       </c>
       <c r="N14">
-        <v>46203</v>
+        <v>46235</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Processo finalizado. Implantação realizada em Agosto.</v>
       </c>
       <c r="P14" t="str">
         <v>Alta</v>
@@ -1026,75 +1111,90 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D15" t="str">
-        <v>Implantação de Telemedicina</v>
+        <v>E-mails corporativos</v>
       </c>
       <c r="E15" t="str">
-        <v>Sistema</v>
+        <v>Emails</v>
       </c>
       <c r="F15" t="str">
         <v>Crítico</v>
       </c>
       <c r="G15" t="str">
-        <v>impacto operacional</v>
+        <v>Comunicação operacional</v>
       </c>
       <c r="H15" t="str">
-        <v>Implantação de Telemedicina (500 minutos)</v>
+        <v>Formalizar contratação das licenças Microsoft e iniciar implantação das contas corporativas.</v>
       </c>
       <c r="I15" t="str">
-        <v>TI</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J15" t="str">
-        <v>Necessidade de investimento para troca de equipamentos</v>
+        <v>Aguardando aprovação orçamentária para regularização das licenças.</v>
       </c>
       <c r="K15">
-        <v>895</v>
+        <v>4141.67</v>
+      </c>
+      <c r="L15">
+        <v>49700</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
       </c>
       <c r="N15">
-        <v>46203</v>
+        <v>46327</v>
+      </c>
+      <c r="O15" t="str">
+        <v/>
       </c>
       <c r="P15" t="str">
-        <v>Alta</v>
+        <v>Média</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>AME Promissão</v>
+        <v>CD Valença</v>
       </c>
       <c r="B16" t="str">
-        <v>São Paulo</v>
+        <v>Piauí</v>
       </c>
       <c r="C16" t="str">
         <v>Urgência e Emergência</v>
       </c>
       <c r="D16" t="str">
-        <v>Emails corporativos</v>
+        <v>Segmentação e segurança da rede Wi-Fi</v>
       </c>
       <c r="E16" t="str">
-        <v>Emails</v>
+        <v>Segurança</v>
       </c>
       <c r="F16" t="str">
-        <v>Crítico</v>
+        <v>Grave</v>
       </c>
       <c r="G16" t="str">
-        <v>Comunicação operacional</v>
+        <v>Risco LGPD</v>
       </c>
       <c r="H16" t="str">
-        <v>Necessidade de contratação dos serviços com a Microsoft</v>
+        <v>Manter a segmentação da rede por VLANs e monitorar os controles de acesso aplicados.</v>
       </c>
       <c r="I16" t="str">
-        <v>TI/Alta Gestão</v>
+        <v>TI</v>
       </c>
       <c r="J16" t="str">
-        <v>Realizado a implantação</v>
+        <v>Concluído</v>
       </c>
       <c r="K16">
-        <v>4141.67</v>
+        <v>0</v>
       </c>
       <c r="L16">
-        <v>49700</v>
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>45962</v>
       </c>
       <c r="N16">
-        <v>46203</v>
+        <v>46207</v>
+      </c>
+      <c r="O16" t="str">
+        <v/>
       </c>
       <c r="P16" t="str">
         <v>Média</v>
@@ -1102,7 +1202,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CD Valença</v>
+        <v>UPA São Raimundo Nonato</v>
       </c>
       <c r="B17" t="str">
         <v>Piauí</v>
@@ -1111,31 +1211,43 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D17" t="str">
-        <v>Controle de segurança Wi-fi</v>
+        <v>PEP não funcional</v>
       </c>
       <c r="E17" t="str">
-        <v>Segurança</v>
+        <v>Prontuario Eletrônico</v>
       </c>
       <c r="F17" t="str">
-        <v>Grave</v>
+        <v>Crítico</v>
       </c>
       <c r="G17" t="str">
-        <v>Risco LGPD</v>
+        <v>Impacto assistencial</v>
       </c>
       <c r="H17" t="str">
-        <v>Criar VLANs</v>
+        <v>Necessidade de apoio do Assistencial sobre uso correto e necessária reimplantação da ferramenta</v>
       </c>
       <c r="I17" t="str">
-        <v>TI</v>
+        <v>Operação</v>
       </c>
       <c r="J17" t="str">
-        <v>Resolvido.</v>
-      </c>
-      <c r="N17">
-        <v>46207</v>
+        <v>Aguardando definição da Secretaria Municipal de Saúde e da área assistencial.</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Definição da SMS</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Ao iniciar dministração da unidade, já existia o sistema</v>
       </c>
       <c r="P17" t="str">
-        <v>Média</v>
+        <v>Alta</v>
       </c>
     </row>
     <row r="18">
@@ -1149,31 +1261,40 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D18" t="str">
-        <v>PEP não funcional</v>
+        <v>Falhas de Wi-Fi</v>
       </c>
       <c r="E18" t="str">
-        <v>Prontuário Eletrônico</v>
+        <v>Rede</v>
       </c>
       <c r="F18" t="str">
         <v>Crítico</v>
       </c>
       <c r="G18" t="str">
-        <v>Impacto assistencial</v>
+        <v>Queda operação</v>
       </c>
       <c r="H18" t="str">
-        <v>Reimplantar sistema</v>
+        <v>Implantar infraestrutura de Wi-Fi para apoio operacional e usuários autorizados.</v>
       </c>
       <c r="I18" t="str">
-        <v>Operação</v>
+        <v>TI</v>
       </c>
       <c r="J18" t="str">
-        <v>Identificado pela TI riscos e repassado para Assistencial, Secretária não responde sobre implantação.</v>
+        <v>Em andamento.</v>
+      </c>
+      <c r="K18">
+        <v>210</v>
+      </c>
+      <c r="L18">
+        <v>1000</v>
+      </c>
+      <c r="M18">
+        <v>46174</v>
       </c>
       <c r="N18">
-        <v>46222</v>
+        <v>46266</v>
       </c>
       <c r="O18" t="str">
-        <v>Ao iniciar Adm já existia o sistema</v>
+        <v/>
       </c>
       <c r="P18" t="str">
         <v>Alta</v>
@@ -1181,7 +1302,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>UPA São Raimundo Nonato</v>
+        <v>CD Picos</v>
       </c>
       <c r="B19" t="str">
         <v>Piauí</v>
@@ -1202,25 +1323,28 @@
         <v>Queda operação</v>
       </c>
       <c r="H19" t="str">
-        <v>Corrigir rede</v>
+        <v>Acompanhar aquisição dos equipamentos previstos em edital e realizar implantação.</v>
       </c>
       <c r="I19" t="str">
-        <v>TI</v>
+        <v>Contratos / TI</v>
       </c>
       <c r="J19" t="str">
-        <v>Unidade não possui wi fi para pacientes.</v>
+        <v>Em processo de contratação por edital.</v>
       </c>
       <c r="K19">
-        <v>210</v>
+        <v>42883.44</v>
       </c>
       <c r="L19">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="M19">
-        <v>46204</v>
+        <v>46113</v>
       </c>
       <c r="N19">
-        <v>46223</v>
+        <v>46296</v>
+      </c>
+      <c r="O19" t="str">
+        <v/>
       </c>
       <c r="P19" t="str">
         <v>Alta</v>
@@ -1237,7 +1361,7 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D20" t="str">
-        <v>Falhas de Wi-Fi</v>
+        <v>Ausência de rede cabeada</v>
       </c>
       <c r="E20" t="str">
         <v>Rede</v>
@@ -1249,22 +1373,28 @@
         <v>Queda operação</v>
       </c>
       <c r="H20" t="str">
-        <v>Corrigir rede</v>
+        <v>Acompanhar execução do processo GC-0228 e implantação da infraestrutura estruturada.</v>
       </c>
       <c r="I20" t="str">
-        <v>Compras</v>
+        <v>Contratos / TI</v>
       </c>
       <c r="J20" t="str">
-        <v>TI solicitou mais equipamentos, processo do edital</v>
+        <v>Em processo de contratação por edital.</v>
       </c>
       <c r="K20">
-        <v>42883.44</v>
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>130000</v>
       </c>
       <c r="M20">
-        <v>46174</v>
+        <v>45962</v>
       </c>
       <c r="N20">
-        <v>46203</v>
+        <v>46266</v>
+      </c>
+      <c r="O20" t="str">
+        <v/>
       </c>
       <c r="P20" t="str">
         <v>Alta</v>
@@ -1272,40 +1402,52 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CD Picos</v>
+        <v>UPA Dr. Thelmo</v>
       </c>
       <c r="B21" t="str">
-        <v>Piauí</v>
+        <v>São Paulo</v>
       </c>
       <c r="C21" t="str">
         <v>Urgência e Emergência</v>
       </c>
       <c r="D21" t="str">
-        <v>Ausência de rede cabeada</v>
+        <v>Lentidão e travamentos</v>
       </c>
       <c r="E21" t="str">
-        <v>Rede</v>
+        <v>Hardware</v>
       </c>
       <c r="F21" t="str">
         <v>Crítico</v>
       </c>
       <c r="G21" t="str">
-        <v>Queda operação</v>
+        <v>Impacto assistencial</v>
       </c>
       <c r="H21" t="str">
-        <v>Corrigir rede</v>
+        <v>Realizar substituição gradual dos equipamentos com baixo desempenho. Pendente 10 equipamentos.</v>
       </c>
       <c r="I21" t="str">
-        <v>Compras</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J21" t="str">
-        <v>Processo de edital no Interact, nº GC-0228</v>
+        <v>Aguardando aprovação orçamentária.</v>
+      </c>
+      <c r="K21">
+        <v>3000</v>
       </c>
       <c r="L21">
-        <v>130000</v>
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>45962</v>
       </c>
       <c r="N21">
-        <v>46295</v>
+        <v>46296</v>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v>Alta</v>
       </c>
     </row>
     <row r="22">
@@ -1319,28 +1461,40 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D22" t="str">
-        <v>Lentidão e travamentos</v>
+        <v>Falhas de Wi-Fi</v>
       </c>
       <c r="E22" t="str">
-        <v>Hardware</v>
+        <v>Rede</v>
       </c>
       <c r="F22" t="str">
         <v>Crítico</v>
       </c>
       <c r="G22" t="str">
-        <v>Impacto assistencial</v>
+        <v>Queda operacional</v>
       </c>
       <c r="H22" t="str">
-        <v>Troca e tuning</v>
+        <v>Implantar melhorias na cobertura da rede sem fio.</v>
       </c>
       <c r="I22" t="str">
         <v>TI</v>
       </c>
       <c r="J22" t="str">
-        <v>Necessidade de investimento para troca de equipamentos</v>
+        <v>Concluído</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>200</v>
+      </c>
+      <c r="M22">
+        <v>45962</v>
       </c>
       <c r="N22">
-        <v>46212</v>
+        <v>46235</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Processo finalizado. Implantação realizada em Agosto.</v>
       </c>
       <c r="P22" t="str">
         <v>Alta</v>
@@ -1348,10 +1502,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>UPA Dr. Thelmo</v>
+        <v>UPA Picos</v>
       </c>
       <c r="B23" t="str">
-        <v>São Paulo</v>
+        <v>Piauí</v>
       </c>
       <c r="C23" t="str">
         <v>Urgência e Emergência</v>
@@ -1369,19 +1523,28 @@
         <v>Queda operacional</v>
       </c>
       <c r="H23" t="str">
-        <v>Ampliar cobertura</v>
+        <v>Executar projeto de ampliação da cobertura para colaboradores e pacientes.</v>
       </c>
       <c r="I23" t="str">
         <v>TI</v>
       </c>
       <c r="J23" t="str">
-        <v>Necessidade de investimento para ampliação de controle</v>
+        <v>Em planejamento.</v>
+      </c>
+      <c r="K23">
+        <v>210</v>
       </c>
       <c r="L23">
-        <v>10000</v>
+        <v>1000</v>
+      </c>
+      <c r="M23">
+        <v>46174</v>
       </c>
       <c r="N23">
-        <v>46203</v>
+        <v>46266</v>
+      </c>
+      <c r="O23" t="str">
+        <v/>
       </c>
       <c r="P23" t="str">
         <v>Alta</v>
@@ -1389,46 +1552,52 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>UPA Picos</v>
+        <v>UPA Tobias Barreto</v>
       </c>
       <c r="B24" t="str">
-        <v>Piauí</v>
+        <v>Sergipe</v>
       </c>
       <c r="C24" t="str">
         <v>Urgência e Emergência</v>
       </c>
       <c r="D24" t="str">
-        <v>Falhas de Wi-Fi</v>
+        <v>Lentidão e travamentos</v>
       </c>
       <c r="E24" t="str">
-        <v>Rede</v>
+        <v>Hardware</v>
       </c>
       <c r="F24" t="str">
         <v>Crítico</v>
       </c>
       <c r="G24" t="str">
-        <v>Queda operacional</v>
+        <v>Impacto assistencial</v>
       </c>
       <c r="H24" t="str">
-        <v>Ampliar cobertura</v>
+        <v>Manter o acompanhamento do desempenho dos equipamentos após as correções realizadas.</v>
       </c>
       <c r="I24" t="str">
         <v>TI</v>
       </c>
       <c r="J24" t="str">
-        <v>Necessidade de investimento para ampliação de controle, Wi fi paciente</v>
+        <v>Concluído</v>
       </c>
       <c r="K24">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="L24">
-        <v>1000</v>
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>46023</v>
       </c>
       <c r="N24">
-        <v>46203</v>
+        <v>46143</v>
+      </c>
+      <c r="O24" t="str">
+        <v/>
       </c>
       <c r="P24" t="str">
-        <v>Alta</v>
+        <v>Média</v>
       </c>
     </row>
     <row r="25">
@@ -1442,25 +1611,40 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D25" t="str">
-        <v>Lentidão e travamentos</v>
+        <v>Link redundante</v>
       </c>
       <c r="E25" t="str">
-        <v>Hardware</v>
+        <v>Performance</v>
       </c>
       <c r="F25" t="str">
         <v>Crítico</v>
       </c>
       <c r="G25" t="str">
-        <v>Impacto assistencial</v>
+        <v>Oscilação de internet</v>
       </c>
       <c r="H25" t="str">
-        <v>Troca e tuning</v>
+        <v>Concluir processo de contratação do segundo link de internet.</v>
       </c>
       <c r="I25" t="str">
         <v>TI</v>
       </c>
       <c r="J25" t="str">
-        <v>Solucionado</v>
+        <v>Em contratação.</v>
+      </c>
+      <c r="K25">
+        <v>400</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>46023</v>
+      </c>
+      <c r="N25">
+        <v>46266</v>
+      </c>
+      <c r="O25" t="str">
+        <v/>
       </c>
       <c r="P25" t="str">
         <v>Média</v>
@@ -1468,40 +1652,49 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>UPA Tobias Barreto</v>
+        <v>UPA Zona Leste Santos</v>
       </c>
       <c r="B26" t="str">
-        <v>Sergipe</v>
+        <v>São Paulo</v>
       </c>
       <c r="C26" t="str">
         <v>Urgência e Emergência</v>
       </c>
       <c r="D26" t="str">
-        <v>Link de internet Redundante</v>
+        <v>Ausência de Wi-Fi Corporativo</v>
       </c>
       <c r="E26" t="str">
-        <v>Performance</v>
+        <v>Infraestrutura</v>
       </c>
       <c r="F26" t="str">
         <v>Crítico</v>
       </c>
       <c r="G26" t="str">
-        <v>Oscilação de internet</v>
+        <v>Limitação de mobilidade</v>
       </c>
       <c r="H26" t="str">
-        <v>Aquisição de novo link</v>
+        <v>Manter o acompanhamento técnico junto à Prefeitura para aprovação e implantação do projeto de Wi-Fi corporativo.</v>
       </c>
       <c r="I26" t="str">
-        <v>TI</v>
+        <v>Alta Gestão / Prefeitura</v>
       </c>
       <c r="J26" t="str">
-        <v>Em processo de contratação</v>
+        <v>Aguardando aprovação da Prefeitura.</v>
       </c>
       <c r="K26">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="L26">
-        <v>300</v>
+        <v>10000</v>
+      </c>
+      <c r="M26">
+        <v>46122</v>
+      </c>
+      <c r="N26" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Enviado relatório técnico</v>
       </c>
       <c r="P26" t="str">
         <v>Média</v>
@@ -1518,7 +1711,7 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D27" t="str">
-        <v>Ausência de Wifi Corporativo</v>
+        <v>Ausência de equipamentos de backup</v>
       </c>
       <c r="E27" t="str">
         <v>Infraestrutura</v>
@@ -1527,54 +1720,84 @@
         <v>Crítico</v>
       </c>
       <c r="G27" t="str">
-        <v>Limitação de mobilidade</v>
+        <v>Parada operacional</v>
       </c>
       <c r="H27" t="str">
-        <v>Implantação de ambiente WIFI</v>
+        <v>Apresentar o estudo técnico e acompanhar a aprovação da Prefeitura para aquisição e implantação dos equipamentos de backup.</v>
       </c>
       <c r="I27" t="str">
-        <v>Montado relatórios técnicos. Necessidade de aprovação da prefeitura.</v>
+        <v>Diretoria / Prefeitura</v>
       </c>
       <c r="J27" t="str">
-        <v>Montado relatório pois processo precisa de aprovação da prefeitura</v>
+        <v>Aguardando aprovação da Prefeitura.</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>5000</v>
+      </c>
+      <c r="M27">
+        <v>46122</v>
+      </c>
+      <c r="N27" t="str">
+        <v>A definir</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Enviado relatório técnico</v>
       </c>
       <c r="P27" t="str">
-        <v>Média</v>
+        <v>Alta</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>UPA Zona Leste Santos</v>
+        <v>CD Teresina</v>
       </c>
       <c r="B28" t="str">
-        <v>São Paulo</v>
+        <v>Piauí</v>
       </c>
       <c r="C28" t="str">
         <v>Urgência e Emergência</v>
       </c>
       <c r="D28" t="str">
-        <v>Ausência de equipamentos de Backup</v>
+        <v>Falhas de Wi-Fi</v>
       </c>
       <c r="E28" t="str">
-        <v>Infraestrutura</v>
+        <v>Rede</v>
       </c>
       <c r="F28" t="str">
         <v>Crítico</v>
       </c>
       <c r="G28" t="str">
-        <v>Parada operacional</v>
+        <v>Queda operacional</v>
       </c>
       <c r="H28" t="str">
-        <v>Processo dependente</v>
+        <v>Implantar expansão da cobertura sem fio.</v>
       </c>
       <c r="I28" t="str">
-        <v>TI/Alta Gestão</v>
+        <v>TI</v>
       </c>
       <c r="J28" t="str">
-        <v>Montado relatórios técnicos. Necessidade de aprovação da prefeitura.</v>
+        <v>Em planejamento.</v>
+      </c>
+      <c r="K28">
+        <v>210</v>
+      </c>
+      <c r="L28">
+        <v>1000</v>
+      </c>
+      <c r="M28">
+        <v>46143</v>
+      </c>
+      <c r="N28">
+        <v>46327</v>
+      </c>
+      <c r="O28" t="str">
+        <v/>
       </c>
       <c r="P28" t="str">
-        <v>Alta</v>
+        <v>Média</v>
       </c>
     </row>
     <row r="29">
@@ -1588,36 +1811,48 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D29" t="str">
-        <v>Falhas de Wi-Fi</v>
+        <v>Implantação de prontuário eletrônico</v>
       </c>
       <c r="E29" t="str">
-        <v>Rede</v>
+        <v>Prontuario Eletrônico</v>
       </c>
       <c r="F29" t="str">
         <v>Crítico</v>
       </c>
       <c r="G29" t="str">
-        <v>Queda operacional</v>
+        <v>Impacto assistencial</v>
       </c>
       <c r="H29" t="str">
-        <v>Ampliar cobertura</v>
+        <v>Concluir levantamento de processos e iniciar implantação com fornecedor.</v>
       </c>
       <c r="I29" t="str">
-        <v>TI</v>
+        <v>TI / Operação</v>
       </c>
       <c r="J29" t="str">
-        <v>Necessidade de investimento para ampliação de controle, Wi fi paciente</v>
+        <v>Em planejamento.</v>
       </c>
       <c r="K29">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="L29">
-        <v>1000</v>
+        <v>0</v>
+      </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29">
+        <v>46296</v>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v>Alta</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>CD Teresina</v>
+        <v>CD Oeiras</v>
       </c>
       <c r="B30" t="str">
         <v>Piauí</v>
@@ -1626,33 +1861,48 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D30" t="str">
-        <v>Implantação de prontuário eletrônico</v>
+        <v>Falhas de Wi-Fi</v>
       </c>
       <c r="E30" t="str">
-        <v>Prontuário Eletrônico</v>
+        <v>Rede</v>
       </c>
       <c r="F30" t="str">
         <v>Crítico</v>
       </c>
       <c r="G30" t="str">
-        <v>Impacto assistencial</v>
+        <v>Queda operacional</v>
       </c>
       <c r="H30" t="str">
-        <v>Implantação de prontuário eletrônico</v>
+        <v>Implantar expansão da cobertura sem fio.</v>
       </c>
       <c r="I30" t="str">
         <v>TI</v>
       </c>
       <c r="J30" t="str">
-        <v>Levantamento de processos junto as áreas e agendamento com fornecedor</v>
+        <v>Em planejamento.</v>
+      </c>
+      <c r="K30">
+        <v>210</v>
+      </c>
+      <c r="L30">
+        <v>1000</v>
+      </c>
+      <c r="M30">
+        <v>46204</v>
       </c>
       <c r="N30">
-        <v>46296</v>
+        <v>46357</v>
+      </c>
+      <c r="O30" t="str">
+        <v/>
+      </c>
+      <c r="P30" t="str">
+        <v>Média</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>CD Oieras</v>
+        <v>CD Oeiras</v>
       </c>
       <c r="B31" t="str">
         <v>Piauí</v>
@@ -1661,73 +1911,148 @@
         <v>Urgência e Emergência</v>
       </c>
       <c r="D31" t="str">
-        <v>Falhas de Wi-Fi</v>
+        <v>Implantação de prontuário eletrônico</v>
       </c>
       <c r="E31" t="str">
-        <v>Rede</v>
+        <v>Prontuário eletronico</v>
       </c>
       <c r="F31" t="str">
         <v>Crítico</v>
       </c>
       <c r="G31" t="str">
-        <v>Queda operacional</v>
+        <v>Impacto assistencial</v>
       </c>
       <c r="H31" t="str">
-        <v>Ampliar cobertura</v>
+        <v>Concluir levantamento de processos e iniciar implantação com fornecedor.</v>
       </c>
       <c r="I31" t="str">
-        <v>TI</v>
+        <v>TI / Operação</v>
       </c>
       <c r="J31" t="str">
-        <v>Necessidade de investimento para ampliação de controle, Wi fi paciente</v>
+        <v>Em planejamento.</v>
       </c>
       <c r="K31">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="L31">
-        <v>1000</v>
+        <v>0</v>
+      </c>
+      <c r="M31">
+        <v>0</v>
+      </c>
+      <c r="N31">
+        <v>46296</v>
+      </c>
+      <c r="O31" t="str">
+        <v/>
+      </c>
+      <c r="P31" t="str">
+        <v>Alta</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>CD Oieras</v>
+        <v>AME CRI</v>
       </c>
       <c r="B32" t="str">
-        <v>Piauí</v>
+        <v>São Paulo</v>
       </c>
       <c r="C32" t="str">
         <v>Urgência e Emergência</v>
       </c>
       <c r="D32" t="str">
-        <v>Implantação de prontuário eletrônico</v>
+        <v>Substituição de impressoras</v>
       </c>
       <c r="E32" t="str">
-        <v>Prontuário Eletrônico</v>
+        <v>Infraestrutura</v>
       </c>
       <c r="F32" t="str">
-        <v>Crítico</v>
+        <v>Grave</v>
       </c>
       <c r="G32" t="str">
-        <v>Impacto assistencial</v>
+        <v>Impacto na continuidade dos serviços de impressão</v>
       </c>
       <c r="H32" t="str">
-        <v>Implantação de prontuário eletrônico</v>
+        <v>Revisar a rubrica orçamentária e as condições do edital, após encerramento sem propostas, para viabilizar nova publicação do processo.</v>
       </c>
       <c r="I32" t="str">
-        <v>TI</v>
+        <v>Alta Gestão</v>
       </c>
       <c r="J32" t="str">
-        <v>Levantamento de processos junto as áreas e agendamento com fornecedor</v>
+        <v>Aguardando revisão orçamentária e nova publicação do edital.</v>
+      </c>
+      <c r="K32">
+        <v>12000</v>
+      </c>
+      <c r="L32">
+        <v>0</v>
+      </c>
+      <c r="M32">
+        <v>46174</v>
       </c>
       <c r="N32">
-        <v>46296</v>
+        <v>46266</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Edital anterior encerrado sem apresentação de propostas.</v>
+      </c>
+      <c r="P32" t="str">
+        <v>Alta</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>UPA Zona Leste Santos</v>
+      </c>
+      <c r="B33" t="str">
+        <v>São Paulo</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Urgência e Emergência</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Substituição de impressoras</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Infraestrutura</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Grave</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Impacto na continuidade dos serviços de impressão</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Revisar a rubrica orçamentária e retomar o processo de contratação para substituição das impressoras da unidade.</v>
+      </c>
+      <c r="I33" t="str">
+        <v>CGI</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Aguardando revisão orçamentária e retomada do edital.</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+      <c r="L33">
+        <v>0</v>
+      </c>
+      <c r="M33">
+        <v>46204</v>
+      </c>
+      <c r="N33">
+        <v>46266</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Processo depende de revisão da rubrica orçamentária.</v>
+      </c>
+      <c r="P33" t="str">
+        <v>Alta</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P33"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>